<commit_message>
Make DMG_EGFR its own subtype, and combine with H3 K28 when K27M is present
Update the crosswalk so DMG_EGFR is DMG, H3 K27-altered, EGFR; tumors that
also carry an H3 K27M/I variant are DMG, H3 K28, EGFR.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
+++ b/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="1084">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="1085">
   <si>
     <t xml:space="preserve">Abbreviation_internal_NIHv3</t>
   </si>
@@ -3264,6 +3264,9 @@
   </si>
   <si>
     <t xml:space="preserve">Control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMG, H3 K27-altered, EGFR</t>
   </si>
 </sst>
 </file>
@@ -5248,7 +5251,7 @@
         <v>302</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>303</v>
+        <v>1084</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">

</xml_diff>

<commit_message>
Rename DMG subtypes to H3 K28-mutant and H3 K28-altered
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
+++ b/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1085" uniqueCount="1085">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="1087">
   <si>
     <t xml:space="preserve">Abbreviation_internal_NIHv3</t>
   </si>
@@ -3267,6 +3267,12 @@
   </si>
   <si>
     <t xml:space="preserve">DMG, H3 K27-altered, EGFR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMG, H3 K28-altered, EGFR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMG, H3 K28-mutant</t>
   </si>
 </sst>
 </file>
@@ -5251,7 +5257,7 @@
         <v>302</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1" t="s">
@@ -5290,7 +5296,7 @@
         <v>309</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>303</v>
+        <v>1086</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="1" t="s">

</xml_diff>

<commit_message>
Prefix HGG, LGG and GNT subtype labels with their family
Rename bare or GBM-prefixed HGG classes (HGAP, HGNET, IHG, GBM MES/RTK),
SEGA and bare GNT in the crosswalk, and map the legacy labels in the
comparison.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
+++ b/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="1087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="1098">
   <si>
     <t xml:space="preserve">Abbreviation_internal_NIHv3</t>
   </si>
@@ -3273,6 +3273,39 @@
   </si>
   <si>
     <t xml:space="preserve">DMG, H3 K28-mutant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GNT, DGONC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GNT, DIG/DIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GNT, DNET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HGG, CBM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HGG, MES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HGG, PNC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GNT, NOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HGG, HGAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HGG, HGNET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HGG, IHG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LGG, SEGA</t>
   </si>
 </sst>
 </file>
@@ -5041,7 +5074,7 @@
         <v>262</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>263</v>
+        <v>1087</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1" t="s">
@@ -5115,7 +5148,7 @@
         <v>277</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>263</v>
+        <v>1088</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1" t="s">
@@ -5333,7 +5366,7 @@
         <v>314</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>263</v>
+        <v>1089</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" s="1" t="s">
@@ -6628,7 +6661,7 @@
         <v>504</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>505</v>
+        <v>1090</v>
       </c>
       <c r="G81" s="1"/>
       <c r="H81" s="1" t="s">
@@ -6665,7 +6698,7 @@
         <v>512</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>513</v>
+        <v>1091</v>
       </c>
       <c r="G82" s="1"/>
       <c r="H82" s="1" t="s">
@@ -6702,7 +6735,7 @@
         <v>519</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>513</v>
+        <v>1091</v>
       </c>
       <c r="G83" s="1"/>
       <c r="H83" s="1" t="s">
@@ -6737,7 +6770,7 @@
         <v>524</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>525</v>
+        <v>1092</v>
       </c>
       <c r="G84" s="1"/>
       <c r="H84" s="1" t="s">
@@ -6772,7 +6805,7 @@
         <v>530</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>531</v>
+        <v>925</v>
       </c>
       <c r="G85" s="1"/>
       <c r="H85" s="1" t="s">
@@ -6807,7 +6840,7 @@
         <v>536</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>531</v>
+        <v>925</v>
       </c>
       <c r="G86" s="1"/>
       <c r="H86" s="1" t="s">
@@ -7023,7 +7056,7 @@
         <v>571</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>263</v>
+        <v>1093</v>
       </c>
       <c r="G92" s="1"/>
       <c r="H92" s="1" t="s">
@@ -7060,7 +7093,7 @@
         <v>577</v>
       </c>
       <c r="F93" s="5" t="s">
-        <v>577</v>
+        <v>1094</v>
       </c>
       <c r="G93" s="1"/>
       <c r="H93" s="1" t="s">
@@ -7095,7 +7128,7 @@
         <v>584</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>585</v>
+        <v>1095</v>
       </c>
       <c r="G94" s="1"/>
       <c r="H94" s="1" t="s">
@@ -7132,7 +7165,7 @@
         <v>591</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>585</v>
+        <v>1095</v>
       </c>
       <c r="G95" s="1"/>
       <c r="H95" s="1" t="s">
@@ -7167,7 +7200,7 @@
         <v>596</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>585</v>
+        <v>1095</v>
       </c>
       <c r="G96" s="1"/>
       <c r="H96" s="1" t="s">
@@ -7241,7 +7274,7 @@
         <v>608</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>608</v>
+        <v>1096</v>
       </c>
       <c r="G98" s="1"/>
       <c r="H98" s="1" t="s">
@@ -10296,7 +10329,7 @@
         <v>1066</v>
       </c>
       <c r="F183" s="1" t="s">
-        <v>1066</v>
+        <v>1097</v>
       </c>
       <c r="G183" s="1"/>
       <c r="H183" s="1" t="s">

</xml_diff>

<commit_message>
Keep spinal subependymoma as EPN, SP-SE (no A/B split)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
+++ b/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="1098">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="1099">
   <si>
     <t xml:space="preserve">Abbreviation_internal_NIHv3</t>
   </si>
@@ -3306,6 +3306,9 @@
   </si>
   <si>
     <t xml:space="preserve">LGG, SEGA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EPN, SP-SE</t>
   </si>
 </sst>
 </file>
@@ -6065,7 +6068,7 @@
         <v>410</v>
       </c>
       <c r="F65" s="5" t="s">
-        <v>411</v>
+        <v>1098</v>
       </c>
       <c r="G65" s="1"/>
       <c r="H65" s="1" t="s">
@@ -6102,7 +6105,7 @@
         <v>418</v>
       </c>
       <c r="F66" s="5" t="s">
-        <v>419</v>
+        <v>1098</v>
       </c>
       <c r="G66" s="1"/>
       <c r="H66" s="1" t="s">

</xml_diff>

<commit_message>
Chordoma naming and manual rows, cranio free-text rule, neurocytoma rule, cell line parent concordance
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
+++ b/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="1099">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="1100">
   <si>
     <t xml:space="preserve">Abbreviation_internal_NIHv3</t>
   </si>
@@ -3309,6 +3309,9 @@
   </si>
   <si>
     <t xml:space="preserve">EPN, SP-SE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHDM</t>
   </si>
 </sst>
 </file>
@@ -4160,7 +4163,7 @@
         <v>100</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>100</v>
+        <v>1099</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1" t="s">

</xml_diff>

<commit_message>
Label DKFZ PA_CORT as LGG, PA ST instead of GNT, MAPK
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
+++ b/analyses/molecular-subtyping-CNS/input/mnp_v12.5_v12.8_NIHv2_v3.1_annotation_with_OPC_subtypes.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="1100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="1101">
   <si>
     <t xml:space="preserve">Abbreviation_internal_NIHv3</t>
   </si>
@@ -3312,6 +3312,9 @@
   </si>
   <si>
     <t xml:space="preserve">CHDM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LGG, PA ST</t>
   </si>
 </sst>
 </file>
@@ -8950,7 +8953,7 @@
         <v>857</v>
       </c>
       <c r="F144" s="5" t="s">
-        <v>291</v>
+        <v>1100</v>
       </c>
       <c r="G144" s="1"/>
       <c r="H144" s="1" t="s">

</xml_diff>